<commit_message>
Update pricing/cost data and dashboard content
Latest edits across SAS/American/Virgin pricing workbooks, batch sheet
recipes, and cost breakdowns, plus refreshed Missions_Operations_Dashboard.html
and minor doc/script touch-ups.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pricing/American/2026.04.09 - 2026 New Contract Pricing-eff 04.08.2026.xlsx
+++ b/Pricing/American/2026.04.09 - 2026 New Contract Pricing-eff 04.08.2026.xlsx
@@ -20960,8 +20960,8 @@
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <TaxCatchAll xmlns="12a9946e-2f22-4d62-9e90-a2605d575b8b" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="700dd037-44e7-4406-9377-bf19ea6f06b3">
+    <TaxCatchAll xmlns="70b03f2f-74c7-4926-a36d-d4bdb9e02d45" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="042478ca-ca2d-4d01-83eb-90396d5625e9">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
@@ -20978,10 +20978,10 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000832148DC42F354DAF29B0D0BBF081E9" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9ba51a3821db048770e807dab2c7edb0">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="700dd037-44e7-4406-9377-bf19ea6f06b3" xmlns:ns3="12a9946e-2f22-4d62-9e90-a2605d575b8b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="222a638a742153f3defe09e7af4707c1" ns2:_="" ns3:_="">
-    <xsd:import namespace="700dd037-44e7-4406-9377-bf19ea6f06b3"/>
-    <xsd:import namespace="12a9946e-2f22-4d62-9e90-a2605d575b8b"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000560CDE7020FBE4F987D5680CBA97CD3" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4fbed0173a2ebcc74ba7d005722587c6">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="042478ca-ca2d-4d01-83eb-90396d5625e9" xmlns:ns3="70b03f2f-74c7-4926-a36d-d4bdb9e02d45" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1e47617018f8bf8a4d157a39e72236d1" ns2:_="" ns3:_="">
+    <xsd:import namespace="042478ca-ca2d-4d01-83eb-90396d5625e9"/>
+    <xsd:import namespace="70b03f2f-74c7-4926-a36d-d4bdb9e02d45"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -20990,17 +20990,13 @@
               <xsd:all>
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
                 <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
                 <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
-                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -21008,7 +21004,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="700dd037-44e7-4406-9377-bf19ea6f06b3" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="042478ca-ca2d-4d01-83eb-90396d5625e9" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -21021,55 +21017,45 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="11" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="c5be1fd7-7535-4a18-99f7-c6c8bb01b25e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="00000000-0000-0000-0000-000000000000" ma:termSetId="00000000-0000-0000-0000-000000000000" ma:anchorId="00000000-0000-0000-0000-000000000000" ma:open="false" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
         </xsd:sequence>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="13" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+    <xsd:element name="MediaServiceEventHashCode" ma:index="15" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="14" nillable="true" ma:displayName="Location" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="15" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="16" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="21" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="12a9946e-2f22-4d62-9e90-a2605d575b8b" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="70b03f2f-74c7-4926-a36d-d4bdb9e02d45" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="12" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{39c7a040-55b6-4baf-bdf7-814612af711d}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="12a9946e-2f22-4d62-9e90-a2605d575b8b">
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{a7cd25fd-8387-47a0-a3a2-f48b21d35c24}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="70b03f2f-74c7-4926-a36d-d4bdb9e02d45">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:MultiChoiceLookup">
@@ -21079,32 +21065,6 @@
           </xsd:extension>
         </xsd:complexContent>
       </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithUsers" ma:index="18" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:UserMulti">
-            <xsd:sequence>
-              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
-                <xsd:complexType>
-                  <xsd:sequence>
-                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
-                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
-                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
-                  </xsd:sequence>
-                </xsd:complexType>
-              </xsd:element>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="19" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -21226,20 +21186,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7692DC86-80C9-4BB5-A37D-1F79B86E84BC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="700dd037-44e7-4406-9377-bf19ea6f06b3"/>
-    <ds:schemaRef ds:uri="12a9946e-2f22-4d62-9e90-a2605d575b8b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DD024E35-EE03-4513-A79D-2AE570A38FBF}"/>
 </file>
</xml_diff>